<commit_message>
update test case sheet
</commit_message>
<xml_diff>
--- a/Unit_Test/TrelloTestCase_QuanPhan.xlsx
+++ b/Unit_Test/TrelloTestCase_QuanPhan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\YPP4-QuanPhan\Unit_Test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F0A8C62-230A-4FB7-819F-A8CBF5FE1D27}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{167AB8E4-2029-43BE-A71B-5BE31F65AB76}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{CF4A998A-5824-4540-835B-D54327114C50}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="125">
   <si>
     <t>Actual Result</t>
   </si>
@@ -385,6 +385,21 @@
   </si>
   <si>
     <t xml:space="preserve"> TC012</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TC024</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TC025</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TC026</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TC027</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TC028</t>
   </si>
 </sst>
 </file>
@@ -1390,19 +1405,29 @@
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
+      <c r="A25" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
+      <c r="A26" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
+      <c r="A27" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="1"/>
+      <c r="A28" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
+      <c r="A29" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="1"/>

</xml_diff>